<commit_message>
Still working on Proper handling of failed, complete and requeued
</commit_message>
<xml_diff>
--- a/autoast/jobs_to_fail.xlsx
+++ b/autoast/jobs_to_fail.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="2985" yWindow="1845" windowWidth="28800" windowHeight="15435" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ast_config" sheetId="1" state="visible" r:id="rId1"/>
@@ -80,7 +80,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -88,9 +88,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
@@ -113,13 +110,7 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
@@ -129,12 +120,38 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
   </cellStyles>
+  <dxfs count="3">
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -213,9 +230,9 @@
   <tableColumns count="14">
     <tableColumn id="1" name="region" totalsRowLabel="Total"/>
     <tableColumn id="2" name="feature_layer"/>
-    <tableColumn id="3" name="crown_file_number"/>
-    <tableColumn id="4" name="disposition_number"/>
-    <tableColumn id="5" name="parcel_number"/>
+    <tableColumn id="3" name="crown_file_number" dataDxfId="2"/>
+    <tableColumn id="4" name="disposition_number" dataDxfId="1"/>
+    <tableColumn id="5" name="parcel_number" dataDxfId="0"/>
     <tableColumn id="6" name="output_directory"/>
     <tableColumn id="7" name="output_directory_same_as_input"/>
     <tableColumn id="8" name="dont_overwrite_outputs"/>
@@ -524,25 +541,25 @@
   <dimension ref="A1:O6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="17.7109375" bestFit="1" customWidth="1" style="11" min="1" max="1"/>
-    <col width="155.140625" bestFit="1" customWidth="1" style="12" min="2" max="2"/>
-    <col width="17.7109375" bestFit="1" customWidth="1" style="13" min="3" max="3"/>
-    <col width="16.85546875" bestFit="1" customWidth="1" style="13" min="4" max="4"/>
-    <col width="17.28515625" bestFit="1" customWidth="1" style="13" min="5" max="5"/>
-    <col width="111.42578125" bestFit="1" customWidth="1" style="11" min="6" max="6"/>
-    <col width="29.28515625" bestFit="1" customWidth="1" style="11" min="7" max="7"/>
-    <col width="20.5703125" bestFit="1" customWidth="1" style="11" min="8" max="8"/>
-    <col width="25.5703125" bestFit="1" customWidth="1" style="11" min="9" max="9"/>
-    <col width="21" bestFit="1" customWidth="1" style="11" min="10" max="10"/>
-    <col width="21.28515625" bestFit="1" customWidth="1" style="11" min="11" max="11"/>
-    <col width="13.7109375" bestFit="1" customWidth="1" style="11" min="12" max="12"/>
-    <col width="14.7109375" bestFit="1" customWidth="1" style="11" min="13" max="13"/>
-    <col width="11.5703125" bestFit="1" customWidth="1" style="14" min="14" max="14"/>
-    <col width="13.5703125" bestFit="1" customWidth="1" style="12" min="15" max="15"/>
+    <col width="17.7109375" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
+    <col width="155.140625" bestFit="1" customWidth="1" style="10" min="2" max="2"/>
+    <col width="17.7109375" bestFit="1" customWidth="1" style="18" min="3" max="3"/>
+    <col width="16.85546875" bestFit="1" customWidth="1" style="18" min="4" max="4"/>
+    <col width="17.28515625" bestFit="1" customWidth="1" style="18" min="5" max="5"/>
+    <col width="111.42578125" bestFit="1" customWidth="1" style="1" min="6" max="6"/>
+    <col width="29.28515625" bestFit="1" customWidth="1" style="1" min="7" max="7"/>
+    <col width="20.5703125" bestFit="1" customWidth="1" style="1" min="8" max="8"/>
+    <col width="25.5703125" bestFit="1" customWidth="1" style="1" min="9" max="9"/>
+    <col width="21" bestFit="1" customWidth="1" style="1" min="10" max="10"/>
+    <col width="21.28515625" bestFit="1" customWidth="1" style="1" min="11" max="11"/>
+    <col width="13.7109375" bestFit="1" customWidth="1" style="1" min="12" max="12"/>
+    <col width="14.7109375" bestFit="1" customWidth="1" style="1" min="13" max="13"/>
+    <col width="11.5703125" bestFit="1" customWidth="1" style="11" min="14" max="14"/>
+    <col width="13.5703125" bestFit="1" customWidth="1" style="10" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="19.5" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>region</t>
         </is>
@@ -552,62 +569,62 @@
           <t>feature_layer</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="15" t="inlineStr">
         <is>
           <t>crown_file_number</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="15" t="inlineStr">
         <is>
           <t>disposition_number</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="15" t="inlineStr">
         <is>
           <t>parcel_number</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>output_directory</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>output_directory_same_as_input</t>
         </is>
       </c>
-      <c r="H1" s="5" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>dont_overwrite_outputs</t>
         </is>
       </c>
-      <c r="I1" s="5" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>skip_conflicts_and_constraints</t>
         </is>
       </c>
-      <c r="J1" s="5" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>suppress_map_creation</t>
         </is>
       </c>
-      <c r="K1" s="5" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>add_maps_to_current</t>
         </is>
       </c>
-      <c r="L1" s="5" t="inlineStr">
+      <c r="L1" s="4" t="inlineStr">
         <is>
           <t>run_as_fcbc</t>
         </is>
       </c>
-      <c r="M1" s="5" t="inlineStr">
+      <c r="M1" s="4" t="inlineStr">
         <is>
           <t>ast_condition</t>
         </is>
       </c>
-      <c r="N1" s="6" t="inlineStr">
+      <c r="N1" s="5" t="inlineStr">
         <is>
           <t>file_number</t>
         </is>
@@ -615,141 +632,141 @@
       <c r="O1" s="2" t="n"/>
     </row>
     <row r="2" ht="19.5" customHeight="1">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Northeast</t>
         </is>
       </c>
-      <c r="B2" s="15" t="inlineStr">
+      <c r="B2" s="12" t="inlineStr">
         <is>
           <t>\\spatialfiles.bcgov\work\srm\nel\Local\Geomatics\Workarea\SharedWork\Northeast_WMU_Bulk_status\AST_TEST\7-55\7-55.shp</t>
         </is>
       </c>
-      <c r="C2" s="8" t="n"/>
-      <c r="D2" s="8" t="n"/>
-      <c r="E2" s="8" t="n"/>
-      <c r="F2" s="7" t="inlineStr">
+      <c r="C2" s="16" t="n"/>
+      <c r="D2" s="16" t="n"/>
+      <c r="E2" s="16" t="n"/>
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>\\spatialfiles.bcgov\work\srm\nel\Local\Geomatics\Workarea\csostad\WildLifePermittingTest\AST_TEST\7-55</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="I2" s="5" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="J2" s="5" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="K2" s="5" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="L2" s="5" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="M2" s="9" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="K2" s="4" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="M2" s="8" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
-      <c r="N2" s="8" t="n"/>
+      <c r="N2" s="7" t="n"/>
       <c r="O2" s="2" t="n"/>
     </row>
     <row r="3" ht="19.5" customHeight="1">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Northeast</t>
         </is>
       </c>
-      <c r="B3" s="15" t="inlineStr">
+      <c r="B3" s="12" t="inlineStr">
         <is>
           <t>\\spatialfiles.bcgov\work\srm\nel\Local\Geomatics\Workarea\SharedWork\Northeast_WMU_Bulk_status\AST_TEST\7-56\7-56.shp</t>
         </is>
       </c>
-      <c r="C3" s="8" t="n"/>
-      <c r="D3" s="8" t="n"/>
-      <c r="E3" s="8" t="n"/>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="C3" s="16" t="n"/>
+      <c r="D3" s="16" t="n"/>
+      <c r="E3" s="16" t="n"/>
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>\\spatialfiles.bcgov\work\srm\nel\Local\Geomatics\Workarea\csostad\WildLifePermittingTest\AST_TEST\7-56</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="J3" s="5" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="K3" s="5" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="L3" s="5" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="M3" s="4" t="inlineStr">
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>Requeued</t>
         </is>
       </c>
-      <c r="N3" s="8" t="n"/>
+      <c r="N3" s="7" t="n"/>
       <c r="O3" s="2" t="n"/>
     </row>
     <row r="4" ht="19.5" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>South_Coast</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="10" t="n">
+      <c r="B4" s="3" t="n"/>
+      <c r="C4" s="14" t="n">
         <v>2411696</v>
       </c>
-      <c r="D4" s="10" t="n">
+      <c r="D4" s="14" t="n">
         <v>923950</v>
       </c>
-      <c r="E4" s="10" t="n">
+      <c r="E4" s="14" t="n">
         <v>968511</v>
       </c>
-      <c r="F4" s="7" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>\\spatialfiles.bcgov\work\srm\nel\Local\Geomatics\Workarea\csostad\WildLifePermittingTest\AST_TEST\Parcel_968511</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>False</t>
         </is>
@@ -759,65 +776,84 @@
           <t>True</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="L4" s="4" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="M4" s="4" t="inlineStr">
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>Requeued</t>
         </is>
       </c>
-      <c r="N4" s="8" t="n"/>
-      <c r="O4" s="4" t="n"/>
+      <c r="N4" s="7" t="n"/>
+      <c r="O4" s="3" t="n"/>
     </row>
     <row r="5" ht="19.5" customHeight="1">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>Northeast</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>\\spatialfiles.bcgov\work\srm\nel\Local\Geomatics\Workarea\csostad\WildLifePermittingTest\ast_test_input_files\895262\895262.shp</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="11" t="n"/>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>\\spatialfiles.bcgov\work\srm\nel\Local\Geomatics\Workarea\csostad\WildLifePermittingTest\ast_test_input_files\895262_1\895262.shp</t>
+        </is>
+      </c>
+      <c r="C5" s="17" t="n"/>
+      <c r="D5" s="17" t="n"/>
+      <c r="E5" s="17" t="n"/>
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="I5" s="5" t="n"/>
-      <c r="J5" s="5" t="n"/>
-      <c r="K5" s="5" t="n"/>
-      <c r="L5" s="5" t="n"/>
-      <c r="M5" s="5" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr">
         <is>
           <t>Requeued</t>
         </is>
       </c>
-      <c r="N5" s="6" t="inlineStr">
+      <c r="N5" s="5" t="inlineStr">
         <is>
           <t>968511_1</t>
         </is>
@@ -825,69 +861,70 @@
       <c r="O5" s="2" t="n"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Northeast</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>\\spatialfiles.bcgov\work\srm\nel\Local\Geomatics\Workarea\csostad\WildLifePermittingTest\ast_test_input_files\876372_v2\ChiefsCabinCreek_50m_buffer.shp</t>
         </is>
       </c>
-      <c r="C6" s="8" t="n"/>
-      <c r="D6" s="8" t="n"/>
-      <c r="E6" s="8" t="n"/>
-      <c r="F6" s="4" t="n"/>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="C6" s="16" t="n"/>
+      <c r="D6" s="16" t="n"/>
+      <c r="E6" s="16" t="n"/>
+      <c r="F6" s="3" t="n"/>
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="I6" s="4" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="J6" s="4" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="K6" s="4" t="inlineStr">
+          <t>False</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
         <is>
           <t>False</t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="M6" s="4" t="inlineStr">
-        <is>
-          <t>Requeued</t>
-        </is>
-      </c>
-      <c r="N6" s="10" t="n">
+          <t>False</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>COMPLETE</t>
+        </is>
+      </c>
+      <c r="N6" s="14" t="n">
         <v>876372</v>
       </c>
-      <c r="O6" s="10" t="n"/>
+      <c r="O6" s="9" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Indexing fixed, now failed and requeud not working
</commit_message>
<xml_diff>
--- a/autoast/jobs_to_fail.xlsx
+++ b/autoast/jobs_to_fail.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>ast_condition</t>
         </is>
       </c>
       <c r="N1" s="4" t="inlineStr">
@@ -632,7 +632,11 @@
           <t>False</t>
         </is>
       </c>
-      <c r="M2" s="1" t="n"/>
+      <c r="M2" s="1" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
       <c r="N2" s="3" t="n"/>
       <c r="O2" s="2" t="n"/>
     </row>
@@ -662,7 +666,7 @@
       </c>
       <c r="H3" s="1" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="I3" s="1" t="inlineStr">
@@ -687,7 +691,7 @@
       </c>
       <c r="M3" s="6" t="inlineStr">
         <is>
-          <t>Queued</t>
+          <t>Requeued</t>
         </is>
       </c>
       <c r="N3" s="3" t="n"/>
@@ -721,7 +725,7 @@
       </c>
       <c r="H4" s="1" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="I4" s="1" t="inlineStr">
@@ -746,7 +750,7 @@
       </c>
       <c r="M4" s="6" t="inlineStr">
         <is>
-          <t>Queued</t>
+          <t>Requeued</t>
         </is>
       </c>
       <c r="N4" s="3" t="n"/>
@@ -774,7 +778,7 @@
       </c>
       <c r="H5" s="1" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="I5" s="1" t="inlineStr">
@@ -799,7 +803,7 @@
       </c>
       <c r="M5" s="6" t="inlineStr">
         <is>
-          <t>Queued</t>
+          <t>Requeued</t>
         </is>
       </c>
       <c r="N5" s="4" t="inlineStr">
@@ -831,7 +835,7 @@
       </c>
       <c r="H6" s="1" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="I6" s="1" t="inlineStr">
@@ -856,7 +860,7 @@
       </c>
       <c r="M6" s="6" t="inlineStr">
         <is>
-          <t>Queued</t>
+          <t>Requeued</t>
         </is>
       </c>
       <c r="N6" s="4" t="n">

</xml_diff>

<commit_message>
- changed "completed" to "Success" Jobs  seem to be running now.
- Load jobs has indexing issue - changed all job_index in load jobs to job_index - 1

Script is running. Last job sits as requed. Logs  show each job failing first, then going to complete
</commit_message>
<xml_diff>
--- a/autoast/jobs_to_fail.xlsx
+++ b/autoast/jobs_to_fail.xlsx
@@ -632,9 +632,9 @@
           <t>False</t>
         </is>
       </c>
-      <c r="M2" s="1" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="M2" s="6" t="inlineStr">
+        <is>
+          <t>COMPLETE</t>
         </is>
       </c>
       <c r="N2" s="3" t="n"/>
@@ -666,7 +666,7 @@
       </c>
       <c r="H3" s="1" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
       <c r="I3" s="1" t="inlineStr">
@@ -691,7 +691,7 @@
       </c>
       <c r="M3" s="6" t="inlineStr">
         <is>
-          <t>Requeued</t>
+          <t>COMPLETE</t>
         </is>
       </c>
       <c r="N3" s="3" t="n"/>
@@ -750,7 +750,7 @@
       </c>
       <c r="M4" s="6" t="inlineStr">
         <is>
-          <t>Requeued</t>
+          <t>COMPLETE</t>
         </is>
       </c>
       <c r="N4" s="3" t="n"/>
@@ -803,7 +803,7 @@
       </c>
       <c r="M5" s="6" t="inlineStr">
         <is>
-          <t>Requeued</t>
+          <t>COMPLETE</t>
         </is>
       </c>
       <c r="N5" s="4" t="inlineStr">

</xml_diff>

<commit_message>
- commented out "continue in line 737 because some of the reque script is not executing
 - Going to remove all references to excel row index. If it doesnt work revert to this point
</commit_message>
<xml_diff>
--- a/autoast/jobs_to_fail.xlsx
+++ b/autoast/jobs_to_fail.xlsx
@@ -3,26 +3,32 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="25596" yWindow="-888" windowWidth="27780" windowHeight="12552" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ast_config" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -36,6 +42,14 @@
       <color rgb="FF000000"/>
       <sz val="11"/>
       <u val="single"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -62,48 +76,87 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
   </cellStyles>
+  <dxfs count="4">
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="bottom"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -177,14 +230,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:N6" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:N6"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:N7" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A1:N7"/>
   <tableColumns count="14">
     <tableColumn id="1" name="region" totalsRowLabel="Total"/>
-    <tableColumn id="2" name="feature_layer"/>
-    <tableColumn id="3" name="crown_file_number"/>
-    <tableColumn id="4" name="disposition_number"/>
-    <tableColumn id="5" name="parcel_number"/>
+    <tableColumn id="2" name="feature_layer" dataDxfId="0"/>
+    <tableColumn id="3" name="crown_file_number" dataDxfId="3"/>
+    <tableColumn id="4" name="disposition_number" dataDxfId="2"/>
+    <tableColumn id="5" name="parcel_number" dataDxfId="1"/>
     <tableColumn id="6" name="output_directory"/>
     <tableColumn id="7" name="output_directory_same_as_input"/>
     <tableColumn id="8" name="dont_overwrite_outputs"/>
@@ -206,10 +259,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="1F497D"/>
@@ -247,71 +300,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -339,7 +392,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -362,11 +415,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -375,13 +428,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -391,7 +444,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -400,7 +453,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -409,7 +462,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -417,10 +470,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -493,21 +546,21 @@
   <dimension ref="A1:O6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="17.71928571428571" bestFit="1" customWidth="1" style="8" min="1" max="1"/>
-    <col width="155.1478571428571" bestFit="1" customWidth="1" style="9" min="2" max="2"/>
-    <col width="17.71928571428571" bestFit="1" customWidth="1" style="10" min="3" max="3"/>
-    <col width="16.86214285714286" bestFit="1" customWidth="1" style="10" min="4" max="4"/>
-    <col width="17.29071428571428" bestFit="1" customWidth="1" style="10" min="5" max="5"/>
-    <col width="111.4335714285714" bestFit="1" customWidth="1" style="8" min="6" max="6"/>
-    <col width="29.29071428571428" bestFit="1" customWidth="1" style="8" min="7" max="7"/>
-    <col width="31.005" bestFit="1" customWidth="1" style="8" min="8" max="8"/>
-    <col width="25.57642857142857" bestFit="1" customWidth="1" style="8" min="9" max="9"/>
-    <col width="21.005" bestFit="1" customWidth="1" style="8" min="10" max="10"/>
-    <col width="21.29071428571428" bestFit="1" customWidth="1" style="8" min="11" max="11"/>
-    <col width="13.71928571428571" bestFit="1" customWidth="1" style="8" min="12" max="12"/>
-    <col width="14.71928571428571" bestFit="1" customWidth="1" style="8" min="13" max="13"/>
-    <col width="11.57642857142857" bestFit="1" customWidth="1" style="11" min="14" max="14"/>
-    <col width="13.57642857142857" bestFit="1" customWidth="1" style="9" min="15" max="15"/>
+    <col width="17.7109375" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
+    <col width="155.140625" bestFit="1" customWidth="1" style="21" min="2" max="2"/>
+    <col width="17.7109375" bestFit="1" customWidth="1" style="17" min="3" max="3"/>
+    <col width="16.85546875" bestFit="1" customWidth="1" style="17" min="4" max="4"/>
+    <col width="17.28515625" bestFit="1" customWidth="1" style="17" min="5" max="5"/>
+    <col width="111.42578125" bestFit="1" customWidth="1" style="1" min="6" max="6"/>
+    <col width="29.28515625" bestFit="1" customWidth="1" style="1" min="7" max="7"/>
+    <col width="20.5703125" bestFit="1" customWidth="1" style="1" min="8" max="8"/>
+    <col width="25.5703125" bestFit="1" customWidth="1" style="1" min="9" max="9"/>
+    <col width="21" bestFit="1" customWidth="1" style="1" min="10" max="10"/>
+    <col width="21.28515625" bestFit="1" customWidth="1" style="1" min="11" max="11"/>
+    <col width="13.7109375" bestFit="1" customWidth="1" style="1" min="12" max="12"/>
+    <col width="14.7109375" bestFit="1" customWidth="1" style="1" min="13" max="13"/>
+    <col width="11.5703125" bestFit="1" customWidth="1" style="11" min="14" max="14"/>
+    <col width="13.5703125" bestFit="1" customWidth="1" style="10" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="19.5" customHeight="1">
@@ -516,67 +569,67 @@
           <t>region</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="18" t="inlineStr">
         <is>
           <t>feature_layer</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="14" t="inlineStr">
         <is>
           <t>crown_file_number</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="14" t="inlineStr">
         <is>
           <t>disposition_number</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="14" t="inlineStr">
         <is>
           <t>parcel_number</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>output_directory</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>output_directory_same_as_input</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>dont_overwrite_outputs</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>skip_conflicts_and_constraints</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>suppress_map_creation</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>add_maps_to_current</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" s="4" t="inlineStr">
         <is>
           <t>run_as_fcbc</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" s="4" t="inlineStr">
         <is>
           <t>ast_condition</t>
         </is>
       </c>
-      <c r="N1" s="4" t="inlineStr">
+      <c r="N1" s="5" t="inlineStr">
         <is>
           <t>file_number</t>
         </is>
@@ -589,55 +642,55 @@
           <t>Northeast</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="19" t="inlineStr">
         <is>
           <t>\\spatialfiles.bcgov\work\srm\nel\Local\Geomatics\Workarea\SharedWork\Northeast_WMU_Bulk_status\AST_TEST\7-55\7-55.shp</t>
         </is>
       </c>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="C2" s="15" t="n"/>
+      <c r="D2" s="15" t="n"/>
+      <c r="E2" s="15" t="n"/>
+      <c r="F2" s="12" t="inlineStr">
         <is>
           <t>\\spatialfiles.bcgov\work\srm\nel\Local\Geomatics\Workarea\csostad\WildLifePermittingTest\AST_TEST\7-55</t>
         </is>
       </c>
-      <c r="G2" s="1" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="H2" s="1" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="I2" s="1" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="J2" s="1" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="K2" s="1" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="L2" s="1" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="M2" s="6" t="inlineStr">
-        <is>
-          <t>COMPLETE</t>
-        </is>
-      </c>
-      <c r="N2" s="3" t="n"/>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="K2" s="4" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="M2" s="8" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="N2" s="7" t="n"/>
       <c r="O2" s="2" t="n"/>
     </row>
     <row r="3" ht="19.5" customHeight="1">
@@ -646,115 +699,115 @@
           <t>Northeast</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="19" t="inlineStr">
         <is>
           <t>\\spatialfiles.bcgov\work\srm\nel\Local\Geomatics\Workarea\SharedWork\Northeast_WMU_Bulk_status\AST_TEST\7-56\7-56.shp</t>
         </is>
       </c>
-      <c r="C3" s="3" t="n"/>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="C3" s="15" t="n"/>
+      <c r="D3" s="15" t="n"/>
+      <c r="E3" s="15" t="n"/>
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>\\spatialfiles.bcgov\work\srm\nel\Local\Geomatics\Workarea\csostad\WildLifePermittingTest\AST_TEST\7-56</t>
         </is>
       </c>
-      <c r="G3" s="1" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="H3" s="1" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="I3" s="1" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="J3" s="1" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="K3" s="1" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="L3" s="1" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="M3" s="6" t="inlineStr">
-        <is>
-          <t>COMPLETE</t>
-        </is>
-      </c>
-      <c r="N3" s="3" t="n"/>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="N3" s="7" t="n"/>
       <c r="O3" s="2" t="n"/>
     </row>
     <row r="4" ht="19.5" customHeight="1">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>South_Coast</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="4" t="n">
+      <c r="B4" s="20" t="n"/>
+      <c r="C4" s="13" t="n">
         <v>2411696</v>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D4" s="13" t="n">
         <v>923950</v>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="E4" s="13" t="n">
         <v>968511</v>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>\\spatialfiles.bcgov\work\srm\nel\Local\Geomatics\Workarea\csostad\WildLifePermittingTest\AST_TEST\Parcel_968511</t>
         </is>
       </c>
-      <c r="G4" s="1" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="H4" s="1" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="I4" s="1" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="J4" s="1" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="K4" s="1" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="L4" s="1" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="M4" s="6" t="inlineStr">
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>COMPLETE</t>
         </is>
       </c>
-      <c r="N4" s="3" t="n"/>
-      <c r="O4" s="1" t="n"/>
+      <c r="N4" s="7" t="n"/>
+      <c r="O4" s="3" t="n"/>
     </row>
     <row r="5" ht="19.5" customHeight="1">
       <c r="A5" s="1" t="inlineStr">
@@ -762,51 +815,50 @@
           <t>Northeast</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="19" t="inlineStr">
         <is>
           <t>\\spatialfiles.bcgov\work\srm\nel\Local\Geomatics\Workarea\csostad\WildLifePermittingTest\ast_test_input_files\895262_1\895262.shp</t>
         </is>
       </c>
-      <c r="C5" s="4" t="n"/>
-      <c r="D5" s="4" t="n"/>
-      <c r="E5" s="4" t="n"/>
-      <c r="F5" s="1" t="n"/>
-      <c r="G5" s="1" t="inlineStr">
+      <c r="C5" s="16" t="n"/>
+      <c r="D5" s="16" t="n"/>
+      <c r="E5" s="16" t="n"/>
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="H5" s="1" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="I5" s="1" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="J5" s="1" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="K5" s="1" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="L5" s="1" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="M5" s="6" t="inlineStr">
-        <is>
-          <t>COMPLETE</t>
-        </is>
-      </c>
-      <c r="N5" s="4" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="N5" s="5" t="inlineStr">
         <is>
           <t>968511_1</t>
         </is>
@@ -814,64 +866,71 @@
       <c r="O5" s="2" t="n"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Northeast</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="19" t="inlineStr">
         <is>
           <t>\\spatialfiles.bcgov\work\srm\nel\Local\Geomatics\Workarea\csostad\WildLifePermittingTest\ast_test_input_files\876372_v2\ChiefsCabinCreek_50m_buffer.shp</t>
         </is>
       </c>
-      <c r="C6" s="3" t="n"/>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="3" t="n"/>
-      <c r="F6" s="1" t="n"/>
-      <c r="G6" s="1" t="inlineStr">
+      <c r="C6" s="15" t="n"/>
+      <c r="D6" s="15" t="n"/>
+      <c r="E6" s="15" t="n"/>
+      <c r="F6" s="3" t="n"/>
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="H6" s="1" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="I6" s="1" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="J6" s="1" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="K6" s="1" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="L6" s="1" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="M6" s="6" t="inlineStr">
-        <is>
-          <t>Requeued</t>
-        </is>
-      </c>
-      <c r="N6" s="4" t="n">
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>COMPLETE</t>
+        </is>
+      </c>
+      <c r="N6" s="13" t="n">
         <v>876372</v>
       </c>
-      <c r="O6" s="4" t="n"/>
+      <c r="O6" s="9" t="n"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added last know config as autoasat_10_18_24
 - autoast version is working worse
</commit_message>
<xml_diff>
--- a/autoast/jobs_to_fail.xlsx
+++ b/autoast/jobs_to_fail.xlsx
@@ -803,7 +803,7 @@
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>COMPLETE</t>
+          <t>Requeued</t>
         </is>
       </c>
       <c r="N4" s="7" t="n"/>
@@ -830,7 +830,7 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -855,7 +855,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>COMPLETE</t>
         </is>
       </c>
       <c r="N5" s="5" t="inlineStr">
@@ -912,7 +912,7 @@
       </c>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>COMPLETE</t>
+          <t>Requeued</t>
         </is>
       </c>
       <c r="N6" s="13" t="n">

</xml_diff>